<commit_message>
Updated ITA_grids model - 2025-09-19 00:54
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06A09013-E97D-4C2D-97D1-57A93A792A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{378868E3-4997-4E2F-852D-D5EE1EDCCE40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="21599" windowHeight="12682" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc" sheetId="7" r:id="rId1"/>
@@ -917,24 +917,66 @@
     <t>pre</t>
   </si>
   <si>
+    <t>distr_solelc_spv_016</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>NRGI</t>
+  </si>
+  <si>
+    <t>daynite</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_015</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 15</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_003</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 3</t>
   </si>
   <si>
-    <t>NRGI</t>
-  </si>
-  <si>
-    <t>daynite</t>
-  </si>
-  <si>
     <t>distr_solelc_spv_018</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 18</t>
   </si>
   <si>
+    <t>distr_solelc_spv_004</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_005</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_022</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 22</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_017</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 17</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_013</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 13</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_002</t>
   </si>
   <si>
@@ -959,10 +1001,52 @@
     <t>connecting solar to buses in cluster 14</t>
   </si>
   <si>
-    <t>distr_solelc_spv_013</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 13</t>
+    <t>distr_solelc_spv_011</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 11</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_024</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 24</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_010</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_012</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 12</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_019</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 19</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_021</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 21</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_023</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 23</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_009</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 9</t>
   </si>
   <si>
     <t>distr_solelc_spv_007</t>
@@ -971,114 +1055,51 @@
     <t>connecting solar to buses in cluster 7</t>
   </si>
   <si>
+    <t>distr_solelc_spv_001</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 1</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_008</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 8</t>
   </si>
   <si>
-    <t>distr_solelc_spv_015</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_001</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_011</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_010</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_012</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_019</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 19</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_004</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_005</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_022</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 22</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_017</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_021</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 21</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_023</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 23</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_024</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 24</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_016</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_009</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 9</t>
-  </si>
-  <si>
     <t>comm-in</t>
   </si>
   <si>
     <t>ncap_cost~USD21_alt</t>
   </si>
   <si>
+    <t>e_w108020416-380,e_w85196861-380,e_w338790588-380,e_w495354824-380,e_w449694943-380,e_IT154-380,e_w1098087457-380,e_w103306951-380,e_w126203383-380,e_w338760116-380,e_w60913666-380</t>
+  </si>
+  <si>
+    <t>e_w321724202-380,e_w103381531-380,e_w103386958-380,e_w418902800-380,e_w145665799-380</t>
+  </si>
+  <si>
     <t>e_w104359058-380,e_IT116-380,e_w103653592-380</t>
   </si>
   <si>
     <t>e_IT40-500,e_IT30-500,e_w84301904-380,e_w82083756-380,e_w59026315-380</t>
   </si>
   <si>
+    <t>e_w104359058-380,e_IT93-380,e_w99694910-380,e_w98902899-380,e_w105153431-380</t>
+  </si>
+  <si>
+    <t>e_IT8-380,e_IT7-380,e_w64200868-380</t>
+  </si>
+  <si>
+    <t>e_w139442467-380,e_w82084013-380,e_IT86-380,e_w81938081-380,e_w155158689-380,e_w59366523-380,e_w158739183-380,e_w81929591-380,e_w100407576-380</t>
+  </si>
+  <si>
+    <t>e_w58992998-380,e_w59462263-380,e_w60725875-380,e_w41892273-400,e_w590522266-380</t>
+  </si>
+  <si>
+    <t>e_w57384507-380,e_w61157826-380,e_w1097982502-380,e_w110138220-380,e_w338753171-380,e_w1117128898-380</t>
+  </si>
+  <si>
     <t>e_w103653592-380,e_w104239352-380,e_w98421779-380,e_w100952845-380,e_w98427149-380,e_w162828577-380</t>
   </si>
   <si>
@@ -1091,58 +1112,103 @@
     <t>e_IT157-380,e_w109993642-380,e_w110310021-380,e_w110330925-380,e_w303965869-380,e_w109588422-380,e_w109756016-380</t>
   </si>
   <si>
-    <t>e_w57384507-380,e_w61157826-380,e_w1097982502-380,e_w110138220-380,e_w338753171-380,e_w1117128898-380</t>
+    <t>e_w255011550-380,e_w303915533-380,e_IT150-380,e_w118987056-380</t>
+  </si>
+  <si>
+    <t>e_IT134-380,e_w339703159-380,e_w40634284-380,e_w81931074-380</t>
+  </si>
+  <si>
+    <t>e_IT149-380,e_w409439916-380,e_w144005863-380,e_w1156702013-380,e_w118987056-380</t>
+  </si>
+  <si>
+    <t>e_w57384507-380,e_IT161-380</t>
+  </si>
+  <si>
+    <t>e_w61626687-380,e_w419423704-380,e_IT140-380,e_r13844905-380,e_w891280888-380,e_w60235685-380,e_w1137611914-380,e_w257351439-380,e_w209982720-380,e_w418565264-380,e_w411026199-380</t>
+  </si>
+  <si>
+    <t>e_w743450089-380,e_w1158716725,e_w58931857-380,e_w76709660-380,e_IT137-380,e_w114661587-380,e_w83872215-380,e_w339706878-380,e_w96190189-380,e_w132450233-380,e_w85196861-380,e_w988654143-380</t>
+  </si>
+  <si>
+    <t>e_IT138-380,e_w74943205-380,e_w143585004-380,e_IT137-380,e_w339706879-380,e_w36873258-380</t>
+  </si>
+  <si>
+    <t>e_w105757794-380,e_w107681459-380,e_w107683818-380,e_w41360305-380,e_w114931087-380</t>
   </si>
   <si>
     <t>e_w100952845-380,e_w107438024-380,e_w236661269-380,e_w105757794-380,e_w116517585-380,e_w211180338-380,e_IT106-380,e_w39255054-380,e_w131291789-380,e_IT108-380,e_w208398923-380,e_w155791516-380</t>
   </si>
   <si>
+    <t>e_IT93-380,e_IT71-380,e_IT72-400,e_w72581705-380,e_IT21-380</t>
+  </si>
+  <si>
     <t>e_w100113593-380,e_IT135-380,e_r4816679-380</t>
   </si>
   <si>
-    <t>e_w321724202-380,e_w103381531-380,e_w103386958-380,e_w418902800-380,e_w145665799-380</t>
-  </si>
-  <si>
-    <t>e_IT93-380,e_IT71-380,e_IT72-400,e_w72581705-380,e_IT21-380</t>
-  </si>
-  <si>
-    <t>e_w255011550-380,e_w303915533-380,e_IT150-380,e_w118987056-380</t>
-  </si>
-  <si>
-    <t>e_IT149-380,e_w409439916-380,e_w144005863-380,e_w1156702013-380,e_w118987056-380</t>
-  </si>
-  <si>
-    <t>e_w57384507-380,e_IT161-380</t>
-  </si>
-  <si>
-    <t>e_w61626687-380,e_w419423704-380,e_IT140-380,e_r13844905-380,e_w891280888-380,e_w60235685-380,e_w1137611914-380,e_w257351439-380,e_w209982720-380,e_w418565264-380,e_w411026199-380</t>
-  </si>
-  <si>
-    <t>e_w104359058-380,e_IT93-380,e_w99694910-380,e_w98902899-380,e_w105153431-380</t>
-  </si>
-  <si>
-    <t>e_IT8-380,e_IT7-380,e_w64200868-380</t>
-  </si>
-  <si>
-    <t>e_w139442467-380,e_w82084013-380,e_IT86-380,e_w81938081-380,e_w155158689-380,e_w59366523-380,e_w158739183-380,e_w81929591-380,e_w100407576-380</t>
-  </si>
-  <si>
-    <t>e_w58992998-380,e_w59462263-380,e_w60725875-380,e_w41892273-400,e_w590522266-380</t>
-  </si>
-  <si>
-    <t>e_w743450089-380,e_w1158716725,e_w58931857-380,e_w76709660-380,e_IT137-380,e_w114661587-380,e_w83872215-380,e_w339706878-380,e_w96190189-380,e_w132450233-380,e_w85196861-380,e_w988654143-380</t>
-  </si>
-  <si>
-    <t>e_IT138-380,e_w74943205-380,e_w143585004-380,e_IT137-380,e_w339706879-380,e_w36873258-380</t>
-  </si>
-  <si>
-    <t>e_IT134-380,e_w339703159-380,e_w40634284-380,e_w81931074-380</t>
-  </si>
-  <si>
-    <t>e_w108020416-380,e_w85196861-380,e_w338790588-380,e_w495354824-380,e_w449694943-380,e_IT154-380,e_w1098087457-380,e_w103306951-380,e_w126203383-380,e_w338760116-380,e_w60913666-380</t>
-  </si>
-  <si>
-    <t>e_w105757794-380,e_w107681459-380,e_w107683818-380,e_w41360305-380,e_w114931087-380</t>
+    <t>distr_wonelc_won_010</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_001</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_014</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_008</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_007</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_013</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 13</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_003</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_006</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_002</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 2</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_004</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_017</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 17</t>
   </si>
   <si>
     <t>distr_wonelc_won_005</t>
@@ -1169,22 +1235,22 @@
     <t>connecting wind onshore to buses in cluster 15</t>
   </si>
   <si>
-    <t>distr_wonelc_won_003</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_006</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_008</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 8</t>
+    <t>distr_wonelc_won_016</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_009</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_019</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 19</t>
   </si>
   <si>
     <t>distr_wonelc_won_012</t>
@@ -1193,70 +1259,70 @@
     <t>connecting wind onshore to buses in cluster 12</t>
   </si>
   <si>
-    <t>distr_wonelc_won_002</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 2</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_004</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_017</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_019</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 19</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_010</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_016</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_009</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_007</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_013</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 13</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_001</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_014</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 14</t>
+    <t>elc_won_010</t>
+  </si>
+  <si>
+    <t>e_w60235685-380,e_w1137611914-380,e_w418565264-380,e_w411026199-380</t>
+  </si>
+  <si>
+    <t>elc_won_001</t>
+  </si>
+  <si>
+    <t>e_w82084013-380,e_w155158689-380,e_w59366523-380,e_w100407576-380,e_w59026315-380,e_w58992998-380,e_w60725875-380</t>
+  </si>
+  <si>
+    <t>elc_won_014</t>
+  </si>
+  <si>
+    <t>e_w743450089-380,e_w76705565-380,e_w1158716725,e_w114661587-380,e_w85196861-380</t>
+  </si>
+  <si>
+    <t>elc_won_008</t>
+  </si>
+  <si>
+    <t>e_w339706879-380,e_w36873258-380,e_r13844905-380</t>
+  </si>
+  <si>
+    <t>elc_won_007</t>
+  </si>
+  <si>
+    <t>e_IT134-380,e_w339703159-380,e_IT138-380,e_w74943205-380</t>
+  </si>
+  <si>
+    <t>elc_won_013</t>
+  </si>
+  <si>
+    <t>e_w108020416-380,e_w110330925-380</t>
+  </si>
+  <si>
+    <t>elc_won_003</t>
+  </si>
+  <si>
+    <t>e_r4816679-380,e_w416989699-380,e_r17467354-380,e_w82762493-380,e_w339706880-380,e_IT141-380</t>
+  </si>
+  <si>
+    <t>elc_won_006</t>
+  </si>
+  <si>
+    <t>e_w40634284-380,e_w81931074-380</t>
+  </si>
+  <si>
+    <t>elc_won_002</t>
+  </si>
+  <si>
+    <t>e_w100113593-380,e_w414663585-380,e_w416989699-380,e_IT135-380</t>
+  </si>
+  <si>
+    <t>elc_won_004</t>
+  </si>
+  <si>
+    <t>e_w103653592-380,e_w100952845-380</t>
+  </si>
+  <si>
+    <t>elc_won_017</t>
+  </si>
+  <si>
+    <t>e_IT161-380,e_w61157826-380,e_w57384507-380,e_w1097982502-380</t>
   </si>
   <si>
     <t>elc_won_005</t>
@@ -1283,22 +1349,22 @@
     <t>e_w255011550-380,e_w303915533-380,e_IT150-380,e_IT149-380,e_w409439916-380,e_w144005863-380,e_w1156702013-380,e_w118987056-380</t>
   </si>
   <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>e_r4816679-380,e_w416989699-380,e_r17467354-380,e_w82762493-380,e_w339706880-380,e_IT141-380</t>
-  </si>
-  <si>
-    <t>elc_won_006</t>
-  </si>
-  <si>
-    <t>e_w40634284-380,e_w81931074-380</t>
-  </si>
-  <si>
-    <t>elc_won_008</t>
-  </si>
-  <si>
-    <t>e_w339706879-380,e_w36873258-380,e_r13844905-380</t>
+    <t>elc_won_016</t>
+  </si>
+  <si>
+    <t>e_w255011550-380,e_w57384507-380,e_w338753171-380</t>
+  </si>
+  <si>
+    <t>elc_won_009</t>
+  </si>
+  <si>
+    <t>e_w81938081-380,e_w143585004-380,e_w158739183-380,e_w81929591-380,e_w74943205-380</t>
+  </si>
+  <si>
+    <t>elc_won_019</t>
+  </si>
+  <si>
+    <t>e_w110138220-380,e_w1103579629-380,e_w109993642-380,e_w110310021-380,e_w303965869-380</t>
   </si>
   <si>
     <t>elc_won_012</t>
@@ -1307,70 +1373,22 @@
     <t>e_w988654143-380,e_w891280888-380,e_w257351439-380,e_w209982720-380,e_IT154-380</t>
   </si>
   <si>
-    <t>elc_won_002</t>
-  </si>
-  <si>
-    <t>e_w100113593-380,e_w414663585-380,e_w416989699-380,e_IT135-380</t>
-  </si>
-  <si>
-    <t>elc_won_004</t>
-  </si>
-  <si>
-    <t>e_w103653592-380,e_w100952845-380</t>
-  </si>
-  <si>
-    <t>elc_won_017</t>
-  </si>
-  <si>
-    <t>e_IT161-380,e_w61157826-380,e_w57384507-380,e_w1097982502-380</t>
-  </si>
-  <si>
-    <t>elc_won_019</t>
-  </si>
-  <si>
-    <t>e_w110138220-380,e_w1103579629-380,e_w109993642-380,e_w110310021-380,e_w303965869-380</t>
-  </si>
-  <si>
-    <t>elc_won_010</t>
-  </si>
-  <si>
-    <t>e_w60235685-380,e_w1137611914-380,e_w418565264-380,e_w411026199-380</t>
-  </si>
-  <si>
-    <t>elc_won_016</t>
-  </si>
-  <si>
-    <t>e_w255011550-380,e_w57384507-380,e_w338753171-380</t>
-  </si>
-  <si>
-    <t>elc_won_009</t>
-  </si>
-  <si>
-    <t>e_w81938081-380,e_w143585004-380,e_w158739183-380,e_w81929591-380,e_w74943205-380</t>
-  </si>
-  <si>
-    <t>elc_won_007</t>
-  </si>
-  <si>
-    <t>e_IT134-380,e_w339703159-380,e_IT138-380,e_w74943205-380</t>
-  </si>
-  <si>
-    <t>elc_won_013</t>
-  </si>
-  <si>
-    <t>e_w108020416-380,e_w110330925-380</t>
-  </si>
-  <si>
-    <t>elc_won_001</t>
-  </si>
-  <si>
-    <t>e_w82084013-380,e_w155158689-380,e_w59366523-380,e_w100407576-380,e_w59026315-380,e_w58992998-380,e_w60725875-380</t>
-  </si>
-  <si>
-    <t>elc_won_014</t>
-  </si>
-  <si>
-    <t>e_w743450089-380,e_w76705565-380,e_w1158716725,e_w114661587-380,e_w85196861-380</t>
+    <t>distr_wofelc_wof_016</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_013</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 13</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_007</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 7</t>
   </si>
   <si>
     <t>distr_wofelc_wof_002</t>
@@ -1379,10 +1397,82 @@
     <t>connecting wind offshore to buses in cluster 2</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_007</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 7</t>
+    <t>distr_wofelc_wof_017</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 17</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_018</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 18</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_014</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_015</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 15</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_012</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 12</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_009</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_008</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_019</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 19</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_006</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_011</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 11</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_001</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_010</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_003</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 3</t>
   </si>
   <si>
     <t>distr_wofelc_wof_004</t>
@@ -1397,94 +1487,22 @@
     <t>connecting wind offshore to buses in cluster 5</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_017</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_011</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_001</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_010</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_003</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_018</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 18</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_014</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_008</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_006</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_015</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_012</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_009</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_016</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_013</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 13</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_019</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 19</t>
+    <t>elc_wof_016</t>
+  </si>
+  <si>
+    <t>e_w303915533-380,e_w203225567,e_w255011550-380,e_IT149-380,e_w118987056-380</t>
+  </si>
+  <si>
+    <t>elc_wof_013</t>
+  </si>
+  <si>
+    <t>e_w110138220-380,e_w85196861-380,e_w1103579629-380</t>
+  </si>
+  <si>
+    <t>elc_wof_007</t>
+  </si>
+  <si>
+    <t>e_w1156702013-380,e_w118987056-380,e_w82767145-380</t>
   </si>
   <si>
     <t>elc_wof_002</t>
@@ -1493,10 +1511,79 @@
     <t>e_w36873258-380</t>
   </si>
   <si>
-    <t>elc_wof_007</t>
-  </si>
-  <si>
-    <t>e_w1156702013-380,e_w118987056-380,e_w82767145-380</t>
+    <t>elc_wof_017</t>
+  </si>
+  <si>
+    <t>e_w57384507-380,e_w338753171-380</t>
+  </si>
+  <si>
+    <t>elc_wof_018</t>
+  </si>
+  <si>
+    <t>e_w57384507-380</t>
+  </si>
+  <si>
+    <t>elc_wof_014</t>
+  </si>
+  <si>
+    <t>e_w57384507-380,e_w61157826-380,e_w110138220-380</t>
+  </si>
+  <si>
+    <t>elc_wof_015</t>
+  </si>
+  <si>
+    <t>e_w255011550-380,e_w118987056-380,e_w57384507-380</t>
+  </si>
+  <si>
+    <t>elc_wof_012</t>
+  </si>
+  <si>
+    <t>e_w743450089-380,e_w114661587-380</t>
+  </si>
+  <si>
+    <t>elc_wof_009</t>
+  </si>
+  <si>
+    <t>e_w100113593-380,e_w414663585-380,e_w416989699-380</t>
+  </si>
+  <si>
+    <t>elc_wof_008</t>
+  </si>
+  <si>
+    <t>e_w82767145-380,e_w416989699-380,e_r17467354-380,e_w82762493-380</t>
+  </si>
+  <si>
+    <t>elc_wof_019</t>
+  </si>
+  <si>
+    <t>elc_wof_006</t>
+  </si>
+  <si>
+    <t>e_w409439916-380,e_w1156702013-380</t>
+  </si>
+  <si>
+    <t>elc_wof_011</t>
+  </si>
+  <si>
+    <t>e_w103653592-380</t>
+  </si>
+  <si>
+    <t>elc_wof_001</t>
+  </si>
+  <si>
+    <t>e_w411026199-380,e_w418565264-380,e_w449694943-380</t>
+  </si>
+  <si>
+    <t>elc_wof_010</t>
+  </si>
+  <si>
+    <t>e_w105757794-380,e_w414663585-380</t>
+  </si>
+  <si>
+    <t>elc_wof_003</t>
+  </si>
+  <si>
+    <t>e_w126203383-380,e_w432729521-380,e_w60913666-380,e_w145665799-380</t>
   </si>
   <si>
     <t>elc_wof_004</t>
@@ -1509,93 +1596,6 @@
   </si>
   <si>
     <t>e_w109756016-380,e_w321724202-380,e_w103381531-380,e_w103386958-380,e_w60888331-380,e_w103386958,e_w145665862-380</t>
-  </si>
-  <si>
-    <t>elc_wof_017</t>
-  </si>
-  <si>
-    <t>e_w57384507-380,e_w338753171-380</t>
-  </si>
-  <si>
-    <t>elc_wof_011</t>
-  </si>
-  <si>
-    <t>e_w103653592-380</t>
-  </si>
-  <si>
-    <t>elc_wof_001</t>
-  </si>
-  <si>
-    <t>e_w411026199-380,e_w418565264-380,e_w449694943-380</t>
-  </si>
-  <si>
-    <t>elc_wof_010</t>
-  </si>
-  <si>
-    <t>e_w105757794-380,e_w414663585-380</t>
-  </si>
-  <si>
-    <t>elc_wof_003</t>
-  </si>
-  <si>
-    <t>e_w126203383-380,e_w432729521-380,e_w60913666-380,e_w145665799-380</t>
-  </si>
-  <si>
-    <t>elc_wof_018</t>
-  </si>
-  <si>
-    <t>e_w57384507-380</t>
-  </si>
-  <si>
-    <t>elc_wof_014</t>
-  </si>
-  <si>
-    <t>e_w57384507-380,e_w61157826-380,e_w110138220-380</t>
-  </si>
-  <si>
-    <t>elc_wof_008</t>
-  </si>
-  <si>
-    <t>e_w82767145-380,e_w416989699-380,e_r17467354-380,e_w82762493-380</t>
-  </si>
-  <si>
-    <t>elc_wof_006</t>
-  </si>
-  <si>
-    <t>e_w409439916-380,e_w1156702013-380</t>
-  </si>
-  <si>
-    <t>elc_wof_015</t>
-  </si>
-  <si>
-    <t>e_w255011550-380,e_w118987056-380,e_w57384507-380</t>
-  </si>
-  <si>
-    <t>elc_wof_012</t>
-  </si>
-  <si>
-    <t>e_w743450089-380,e_w114661587-380</t>
-  </si>
-  <si>
-    <t>elc_wof_009</t>
-  </si>
-  <si>
-    <t>e_w100113593-380,e_w414663585-380,e_w416989699-380</t>
-  </si>
-  <si>
-    <t>elc_wof_016</t>
-  </si>
-  <si>
-    <t>e_w303915533-380,e_w203225567,e_w255011550-380,e_IT149-380,e_w118987056-380</t>
-  </si>
-  <si>
-    <t>elc_wof_013</t>
-  </si>
-  <si>
-    <t>e_w110138220-380,e_w85196861-380,e_w1103579629-380</t>
-  </si>
-  <si>
-    <t>elc_wof_019</t>
   </si>
   <si>
     <t>e_won_001</t>
@@ -6868,7 +6868,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAC1152C-3F66-4155-A929-667434261FD4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF1B3FF-9CD1-4296-BF17-4580B7EAD8BF}">
   <dimension ref="B9:BD34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7106,16 +7106,16 @@
         <v>262</v>
       </c>
       <c r="Y11" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="Z11" t="s">
         <v>314</v>
       </c>
       <c r="AA11">
-        <v>0.99736118721915257</v>
+        <v>0.99832448937819496</v>
       </c>
       <c r="AB11">
-        <v>48.378234315535408</v>
+        <v>30.717694733092841</v>
       </c>
       <c r="AD11" t="s">
         <v>261</v>
@@ -7148,10 +7148,10 @@
         <v>377</v>
       </c>
       <c r="AO11">
-        <v>0.99845919630435342</v>
+        <v>0.99874953222888541</v>
       </c>
       <c r="AP11">
-        <v>28.248067753520438</v>
+        <v>22.925242470433936</v>
       </c>
       <c r="AR11" t="s">
         <v>261</v>
@@ -7184,10 +7184,10 @@
         <v>453</v>
       </c>
       <c r="BC11">
-        <v>0.99300217097749499</v>
+        <v>0.99519711687725765</v>
       </c>
       <c r="BD11">
-        <v>128.29353207925857</v>
+        <v>88.052857250275622</v>
       </c>
     </row>
     <row r="12" spans="2:56">
@@ -7252,16 +7252,16 @@
         <v>266</v>
       </c>
       <c r="Y12" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="Z12" t="s">
         <v>315</v>
       </c>
       <c r="AA12">
-        <v>0.99856694466146878</v>
+        <v>0.99846319033655173</v>
       </c>
       <c r="AB12">
-        <v>26.272681206405</v>
+        <v>28.174843829885099</v>
       </c>
       <c r="AD12" t="s">
         <v>261</v>
@@ -7294,10 +7294,10 @@
         <v>379</v>
       </c>
       <c r="AO12">
-        <v>0.99882321467857593</v>
+        <v>0.99918091147922183</v>
       </c>
       <c r="AP12">
-        <v>21.574397559441575</v>
+        <v>15.016622880933385</v>
       </c>
       <c r="AR12" t="s">
         <v>261</v>
@@ -7330,10 +7330,10 @@
         <v>455</v>
       </c>
       <c r="BC12">
-        <v>0.99135720783404546</v>
+        <v>0.99511895269233019</v>
       </c>
       <c r="BD12">
-        <v>158.45118970916684</v>
+        <v>89.485867307280429</v>
       </c>
     </row>
     <row r="13" spans="2:56">
@@ -7398,16 +7398,16 @@
         <v>268</v>
       </c>
       <c r="Y13" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Z13" t="s">
         <v>316</v>
       </c>
       <c r="AA13">
-        <v>0.99860660541325685</v>
+        <v>0.99736118721915257</v>
       </c>
       <c r="AB13">
-        <v>25.545567423624604</v>
+        <v>48.378234315535408</v>
       </c>
       <c r="AD13" t="s">
         <v>261</v>
@@ -7440,10 +7440,10 @@
         <v>381</v>
       </c>
       <c r="AO13">
-        <v>0.99838829169023302</v>
+        <v>0.99876840171930181</v>
       </c>
       <c r="AP13">
-        <v>29.547985679061497</v>
+        <v>22.579301812799098</v>
       </c>
       <c r="AR13" t="s">
         <v>261</v>
@@ -7476,10 +7476,10 @@
         <v>457</v>
       </c>
       <c r="BC13">
-        <v>0.99689089953602861</v>
+        <v>0.99135720783404546</v>
       </c>
       <c r="BD13">
-        <v>57.000175172809875</v>
+        <v>158.45118970916684</v>
       </c>
     </row>
     <row r="14" spans="2:56">
@@ -7544,16 +7544,16 @@
         <v>270</v>
       </c>
       <c r="Y14" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="Z14" t="s">
         <v>317</v>
       </c>
       <c r="AA14">
-        <v>0.99930680862803622</v>
+        <v>0.99856694466146878</v>
       </c>
       <c r="AB14">
-        <v>12.708508486002591</v>
+        <v>26.272681206405</v>
       </c>
       <c r="AD14" t="s">
         <v>261</v>
@@ -7586,10 +7586,10 @@
         <v>383</v>
       </c>
       <c r="AO14">
-        <v>0.99665930146480552</v>
+        <v>0.99831790956100308</v>
       </c>
       <c r="AP14">
-        <v>61.246139811898914</v>
+        <v>30.838324714942974</v>
       </c>
       <c r="AR14" t="s">
         <v>261</v>
@@ -7622,10 +7622,10 @@
         <v>459</v>
       </c>
       <c r="BC14">
-        <v>0.99657569928293988</v>
+        <v>0.99300217097749499</v>
       </c>
       <c r="BD14">
-        <v>62.778846479435288</v>
+        <v>128.29353207925857</v>
       </c>
     </row>
     <row r="15" spans="2:56">
@@ -7690,16 +7690,16 @@
         <v>272</v>
       </c>
       <c r="Y15" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="Z15" t="s">
         <v>318</v>
       </c>
       <c r="AA15">
-        <v>0.99873146688652226</v>
+        <v>0.99877722064413432</v>
       </c>
       <c r="AB15">
-        <v>23.256440413758234</v>
+        <v>22.417621524203621</v>
       </c>
       <c r="AD15" t="s">
         <v>261</v>
@@ -7732,10 +7732,10 @@
         <v>385</v>
       </c>
       <c r="AO15">
-        <v>0.99833657244056218</v>
+        <v>0.99666227090030635</v>
       </c>
       <c r="AP15">
-        <v>30.496171923027788</v>
+        <v>61.191700161050683</v>
       </c>
       <c r="AR15" t="s">
         <v>261</v>
@@ -7836,16 +7836,16 @@
         <v>274</v>
       </c>
       <c r="Y16" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="Z16" t="s">
         <v>319</v>
       </c>
       <c r="AA16">
-        <v>0.99875191609374314</v>
+        <v>0.99600892100673577</v>
       </c>
       <c r="AB16">
-        <v>22.881538281374802</v>
+        <v>73.169781543177265</v>
       </c>
       <c r="AD16" t="s">
         <v>261</v>
@@ -7878,10 +7878,10 @@
         <v>387</v>
       </c>
       <c r="AO16">
-        <v>0.99791596742605326</v>
+        <v>0.99709123993747251</v>
       </c>
       <c r="AP16">
-        <v>38.207263855690094</v>
+        <v>53.327267813004184</v>
       </c>
       <c r="AR16" t="s">
         <v>261</v>
@@ -7914,10 +7914,10 @@
         <v>463</v>
       </c>
       <c r="BC16">
-        <v>0.99706526987313149</v>
+        <v>0.98395626279590787</v>
       </c>
       <c r="BD16">
-        <v>53.8033856592563</v>
+        <v>294.13518207502182</v>
       </c>
     </row>
     <row r="17" spans="2:56">
@@ -7982,16 +7982,16 @@
         <v>276</v>
       </c>
       <c r="Y17" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="Z17" t="s">
         <v>320</v>
       </c>
       <c r="AA17">
-        <v>0.99748803033916245</v>
+        <v>0.9992072598548265</v>
       </c>
       <c r="AB17">
-        <v>46.052777115354985</v>
+        <v>14.533569328181747</v>
       </c>
       <c r="AD17" t="s">
         <v>261</v>
@@ -8024,10 +8024,10 @@
         <v>389</v>
       </c>
       <c r="AO17">
-        <v>0.99831790956100308</v>
+        <v>0.99833657244056218</v>
       </c>
       <c r="AP17">
-        <v>30.838324714942974</v>
+        <v>30.496171923027788</v>
       </c>
       <c r="AR17" t="s">
         <v>261</v>
@@ -8060,10 +8060,10 @@
         <v>465</v>
       </c>
       <c r="BC17">
-        <v>0.99447806844329845</v>
+        <v>0.98404695622985239</v>
       </c>
       <c r="BD17">
-        <v>101.23541187286283</v>
+        <v>292.47246911937344</v>
       </c>
     </row>
     <row r="18" spans="2:56">
@@ -8128,16 +8128,16 @@
         <v>278</v>
       </c>
       <c r="Y18" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="Z18" t="s">
         <v>321</v>
       </c>
       <c r="AA18">
-        <v>0.99908657148051871</v>
+        <v>0.99886825748232866</v>
       </c>
       <c r="AB18">
-        <v>16.746189523824366</v>
+        <v>20.748612823974995</v>
       </c>
       <c r="AD18" t="s">
         <v>261</v>
@@ -8170,10 +8170,10 @@
         <v>391</v>
       </c>
       <c r="AO18">
-        <v>0.9990306565657765</v>
+        <v>0.99791596742605326</v>
       </c>
       <c r="AP18">
-        <v>17.771296294096938</v>
+        <v>38.207263855690094</v>
       </c>
       <c r="AR18" t="s">
         <v>261</v>
@@ -8206,10 +8206,10 @@
         <v>467</v>
       </c>
       <c r="BC18">
-        <v>0.99517233046898579</v>
+        <v>0.98457979899191617</v>
       </c>
       <c r="BD18">
-        <v>88.507274735259927</v>
+        <v>282.70368514820279</v>
       </c>
     </row>
     <row r="19" spans="2:56">
@@ -8274,16 +8274,16 @@
         <v>280</v>
       </c>
       <c r="Y19" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="Z19" t="s">
         <v>322</v>
       </c>
       <c r="AA19">
-        <v>0.99797368969783629</v>
+        <v>0.99748803033916245</v>
       </c>
       <c r="AB19">
-        <v>37.149022206335331</v>
+        <v>46.052777115354985</v>
       </c>
       <c r="AD19" t="s">
         <v>261</v>
@@ -8352,10 +8352,10 @@
         <v>469</v>
       </c>
       <c r="BC19">
-        <v>0.99560743175223188</v>
+        <v>0.99601718841685227</v>
       </c>
       <c r="BD19">
-        <v>80.530417875749265</v>
+        <v>73.018212357708393</v>
       </c>
     </row>
     <row r="20" spans="2:56">
@@ -8420,16 +8420,16 @@
         <v>282</v>
       </c>
       <c r="Y20" t="s">
-        <v>250</v>
+        <v>237</v>
       </c>
       <c r="Z20" t="s">
         <v>323</v>
       </c>
       <c r="AA20">
-        <v>0.99846319033655173</v>
+        <v>0.99860660541325685</v>
       </c>
       <c r="AB20">
-        <v>28.174843829885099</v>
+        <v>25.545567423624604</v>
       </c>
       <c r="AD20" t="s">
         <v>261</v>
@@ -8498,10 +8498,10 @@
         <v>471</v>
       </c>
       <c r="BC20">
-        <v>0.98395626279590787</v>
+        <v>0.9951563190122551</v>
       </c>
       <c r="BD20">
-        <v>294.13518207502182</v>
+        <v>88.800818108657467</v>
       </c>
     </row>
     <row r="21" spans="2:56">
@@ -8566,16 +8566,16 @@
         <v>284</v>
       </c>
       <c r="Y21" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="Z21" t="s">
         <v>324</v>
       </c>
       <c r="AA21">
-        <v>0.99911795750826049</v>
+        <v>0.99930680862803622</v>
       </c>
       <c r="AB21">
-        <v>16.170779015225147</v>
+        <v>12.708508486002591</v>
       </c>
       <c r="AD21" t="s">
         <v>261</v>
@@ -8644,10 +8644,10 @@
         <v>473</v>
       </c>
       <c r="BC21">
-        <v>0.98404695622985239</v>
+        <v>0.99680123445612556</v>
       </c>
       <c r="BD21">
-        <v>292.47246911937344</v>
+        <v>58.644034971032312</v>
       </c>
     </row>
     <row r="22" spans="2:56">
@@ -8712,16 +8712,16 @@
         <v>286</v>
       </c>
       <c r="Y22" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="Z22" t="s">
         <v>325</v>
       </c>
       <c r="AA22">
-        <v>0.99352392397859468</v>
+        <v>0.99873146688652226</v>
       </c>
       <c r="AB22">
-        <v>118.7280603924299</v>
+        <v>23.256440413758234</v>
       </c>
       <c r="AD22" t="s">
         <v>261</v>
@@ -8754,10 +8754,10 @@
         <v>399</v>
       </c>
       <c r="AO22">
-        <v>0.99824223632994047</v>
+        <v>0.99845919630435342</v>
       </c>
       <c r="AP22">
-        <v>32.225667284425562</v>
+        <v>28.248067753520438</v>
       </c>
       <c r="AR22" t="s">
         <v>261</v>
@@ -8787,13 +8787,13 @@
         <v>474</v>
       </c>
       <c r="BB22" t="s">
-        <v>475</v>
+        <v>463</v>
       </c>
       <c r="BC22">
-        <v>0.99680123445612556</v>
+        <v>0.98532533439704995</v>
       </c>
       <c r="BD22">
-        <v>58.644034971032312</v>
+        <v>269.0355360540841</v>
       </c>
     </row>
     <row r="23" spans="2:56">
@@ -8858,16 +8858,16 @@
         <v>288</v>
       </c>
       <c r="Y23" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="Z23" t="s">
         <v>326</v>
       </c>
       <c r="AA23">
-        <v>0.99660728585884595</v>
+        <v>0.99875191609374314</v>
       </c>
       <c r="AB23">
-        <v>62.199759254490814</v>
+        <v>22.881538281374802</v>
       </c>
       <c r="AD23" t="s">
         <v>261</v>
@@ -8900,10 +8900,10 @@
         <v>401</v>
       </c>
       <c r="AO23">
-        <v>0.99874953222888541</v>
+        <v>0.99882321467857593</v>
       </c>
       <c r="AP23">
-        <v>22.925242470433936</v>
+        <v>21.574397559441575</v>
       </c>
       <c r="AR23" t="s">
         <v>261</v>
@@ -8930,10 +8930,10 @@
         <v>438</v>
       </c>
       <c r="BA23" t="s">
+        <v>475</v>
+      </c>
+      <c r="BB23" t="s">
         <v>476</v>
-      </c>
-      <c r="BB23" t="s">
-        <v>477</v>
       </c>
       <c r="BC23">
         <v>0.99661535764871823</v>
@@ -9004,16 +9004,16 @@
         <v>290</v>
       </c>
       <c r="Y24" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="Z24" t="s">
         <v>327</v>
       </c>
       <c r="AA24">
-        <v>0.98702432691207775</v>
+        <v>0.99352392397859468</v>
       </c>
       <c r="AB24">
-        <v>237.88733994524034</v>
+        <v>118.7280603924299</v>
       </c>
       <c r="AD24" t="s">
         <v>261</v>
@@ -9046,10 +9046,10 @@
         <v>403</v>
       </c>
       <c r="AO24">
-        <v>0.99117946235007082</v>
+        <v>0.99838829169023302</v>
       </c>
       <c r="AP24">
-        <v>161.7098569153674</v>
+        <v>29.547985679061497</v>
       </c>
       <c r="AR24" t="s">
         <v>261</v>
@@ -9076,16 +9076,16 @@
         <v>440</v>
       </c>
       <c r="BA24" t="s">
+        <v>477</v>
+      </c>
+      <c r="BB24" t="s">
         <v>478</v>
       </c>
-      <c r="BB24" t="s">
-        <v>479</v>
-      </c>
       <c r="BC24">
-        <v>0.98457979899191617</v>
+        <v>0.99706526987313149</v>
       </c>
       <c r="BD24">
-        <v>282.70368514820279</v>
+        <v>53.8033856592563</v>
       </c>
     </row>
     <row r="25" spans="2:56">
@@ -9150,16 +9150,16 @@
         <v>292</v>
       </c>
       <c r="Y25" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="Z25" t="s">
         <v>328</v>
       </c>
       <c r="AA25">
-        <v>0.99897502886966327</v>
+        <v>0.99749418850407234</v>
       </c>
       <c r="AB25">
-        <v>18.791137389507082</v>
+        <v>45.939877425340249</v>
       </c>
       <c r="AD25" t="s">
         <v>261</v>
@@ -9192,10 +9192,10 @@
         <v>405</v>
       </c>
       <c r="AO25">
-        <v>0.99872153620715554</v>
+        <v>0.99665930146480552</v>
       </c>
       <c r="AP25">
-        <v>23.438502868816123</v>
+        <v>61.246139811898914</v>
       </c>
       <c r="AR25" t="s">
         <v>261</v>
@@ -9222,16 +9222,16 @@
         <v>442</v>
       </c>
       <c r="BA25" t="s">
+        <v>479</v>
+      </c>
+      <c r="BB25" t="s">
         <v>480</v>
       </c>
-      <c r="BB25" t="s">
-        <v>481</v>
-      </c>
       <c r="BC25">
-        <v>0.99601718841685227</v>
+        <v>0.99447806844329845</v>
       </c>
       <c r="BD25">
-        <v>73.018212357708393</v>
+        <v>101.23541187286283</v>
       </c>
     </row>
     <row r="26" spans="2:56">
@@ -9296,16 +9296,16 @@
         <v>294</v>
       </c>
       <c r="Y26" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="Z26" t="s">
         <v>329</v>
       </c>
       <c r="AA26">
-        <v>0.99877722064413432</v>
+        <v>0.99660728585884595</v>
       </c>
       <c r="AB26">
-        <v>22.417621524203621</v>
+        <v>62.199759254490814</v>
       </c>
       <c r="AD26" t="s">
         <v>261</v>
@@ -9338,10 +9338,10 @@
         <v>407</v>
       </c>
       <c r="AO26">
-        <v>0.99666227090030635</v>
+        <v>0.99117946235007082</v>
       </c>
       <c r="AP26">
-        <v>61.191700161050683</v>
+        <v>161.7098569153674</v>
       </c>
       <c r="AR26" t="s">
         <v>261</v>
@@ -9368,16 +9368,16 @@
         <v>444</v>
       </c>
       <c r="BA26" t="s">
+        <v>481</v>
+      </c>
+      <c r="BB26" t="s">
         <v>482</v>
       </c>
-      <c r="BB26" t="s">
-        <v>483</v>
-      </c>
       <c r="BC26">
-        <v>0.9951563190122551</v>
+        <v>0.99517233046898579</v>
       </c>
       <c r="BD26">
-        <v>88.800818108657467</v>
+        <v>88.507274735259927</v>
       </c>
     </row>
     <row r="27" spans="2:56">
@@ -9442,16 +9442,16 @@
         <v>296</v>
       </c>
       <c r="Y27" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="Z27" t="s">
         <v>330</v>
       </c>
       <c r="AA27">
-        <v>0.99600892100673577</v>
+        <v>0.98702432691207775</v>
       </c>
       <c r="AB27">
-        <v>73.169781543177265</v>
+        <v>237.88733994524034</v>
       </c>
       <c r="AD27" t="s">
         <v>261</v>
@@ -9484,10 +9484,10 @@
         <v>409</v>
       </c>
       <c r="AO27">
-        <v>0.99709123993747251</v>
+        <v>0.99872153620715554</v>
       </c>
       <c r="AP27">
-        <v>53.327267813004184</v>
+        <v>23.438502868816123</v>
       </c>
       <c r="AR27" t="s">
         <v>261</v>
@@ -9514,16 +9514,16 @@
         <v>446</v>
       </c>
       <c r="BA27" t="s">
+        <v>483</v>
+      </c>
+      <c r="BB27" t="s">
         <v>484</v>
       </c>
-      <c r="BB27" t="s">
-        <v>485</v>
-      </c>
       <c r="BC27">
-        <v>0.99519711687725765</v>
+        <v>0.99560743175223188</v>
       </c>
       <c r="BD27">
-        <v>88.052857250275622</v>
+        <v>80.530417875749265</v>
       </c>
     </row>
     <row r="28" spans="2:56">
@@ -9588,16 +9588,16 @@
         <v>298</v>
       </c>
       <c r="Y28" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="Z28" t="s">
         <v>331</v>
       </c>
       <c r="AA28">
-        <v>0.9992072598548265</v>
+        <v>0.99897502886966327</v>
       </c>
       <c r="AB28">
-        <v>14.533569328181747</v>
+        <v>18.791137389507082</v>
       </c>
       <c r="AD28" t="s">
         <v>261</v>
@@ -9630,10 +9630,10 @@
         <v>411</v>
       </c>
       <c r="AO28">
-        <v>0.99918091147922183</v>
+        <v>0.99824223632994047</v>
       </c>
       <c r="AP28">
-        <v>15.016622880933385</v>
+        <v>32.225667284425562</v>
       </c>
       <c r="AR28" t="s">
         <v>261</v>
@@ -9660,16 +9660,16 @@
         <v>448</v>
       </c>
       <c r="BA28" t="s">
+        <v>485</v>
+      </c>
+      <c r="BB28" t="s">
         <v>486</v>
       </c>
-      <c r="BB28" t="s">
-        <v>487</v>
-      </c>
       <c r="BC28">
-        <v>0.99511895269233019</v>
+        <v>0.99689089953602861</v>
       </c>
       <c r="BD28">
-        <v>89.485867307280429</v>
+        <v>57.000175172809875</v>
       </c>
     </row>
     <row r="29" spans="2:56">
@@ -9734,16 +9734,16 @@
         <v>300</v>
       </c>
       <c r="Y29" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="Z29" t="s">
         <v>332</v>
       </c>
       <c r="AA29">
-        <v>0.99886825748232866</v>
+        <v>0.99837547744095589</v>
       </c>
       <c r="AB29">
-        <v>20.748612823974995</v>
+        <v>29.782913582474833</v>
       </c>
       <c r="AD29" t="s">
         <v>261</v>
@@ -9776,10 +9776,10 @@
         <v>413</v>
       </c>
       <c r="AO29">
-        <v>0.99876840171930181</v>
+        <v>0.9990306565657765</v>
       </c>
       <c r="AP29">
-        <v>22.579301812799098</v>
+        <v>17.771296294096938</v>
       </c>
       <c r="AR29" t="s">
         <v>261</v>
@@ -9806,16 +9806,16 @@
         <v>450</v>
       </c>
       <c r="BA29" t="s">
+        <v>487</v>
+      </c>
+      <c r="BB29" t="s">
         <v>488</v>
       </c>
-      <c r="BB29" t="s">
-        <v>471</v>
-      </c>
       <c r="BC29">
-        <v>0.98532533439704995</v>
+        <v>0.99657569928293988</v>
       </c>
       <c r="BD29">
-        <v>269.0355360540841</v>
+        <v>62.778846479435288</v>
       </c>
     </row>
     <row r="30" spans="2:56">
@@ -9880,16 +9880,16 @@
         <v>302</v>
       </c>
       <c r="Y30" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="Z30" t="s">
         <v>333</v>
       </c>
       <c r="AA30">
-        <v>0.99837547744095589</v>
+        <v>0.99803201804692143</v>
       </c>
       <c r="AB30">
-        <v>29.782913582474833</v>
+        <v>36.079669139774055</v>
       </c>
     </row>
     <row r="31" spans="2:56">
@@ -9954,16 +9954,16 @@
         <v>304</v>
       </c>
       <c r="Y31" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="Z31" t="s">
         <v>334</v>
       </c>
       <c r="AA31">
-        <v>0.99803201804692143</v>
+        <v>0.99839748836760267</v>
       </c>
       <c r="AB31">
-        <v>36.079669139774055</v>
+        <v>29.37937992728429</v>
       </c>
     </row>
     <row r="32" spans="2:56">
@@ -10028,16 +10028,16 @@
         <v>306</v>
       </c>
       <c r="Y32" t="s">
-        <v>259</v>
+        <v>242</v>
       </c>
       <c r="Z32" t="s">
         <v>335</v>
       </c>
       <c r="AA32">
-        <v>0.99749418850407234</v>
+        <v>0.99908657148051871</v>
       </c>
       <c r="AB32">
-        <v>45.939877425340249</v>
+        <v>16.746189523824366</v>
       </c>
     </row>
     <row r="33" spans="2:28">
@@ -10102,16 +10102,16 @@
         <v>308</v>
       </c>
       <c r="Y33" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="Z33" t="s">
         <v>336</v>
       </c>
       <c r="AA33">
-        <v>0.99832448937819496</v>
+        <v>0.99911795750826049</v>
       </c>
       <c r="AB33">
-        <v>30.717694733092841</v>
+        <v>16.170779015225147</v>
       </c>
     </row>
     <row r="34" spans="2:28">
@@ -10176,16 +10176,16 @@
         <v>310</v>
       </c>
       <c r="Y34" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Z34" t="s">
         <v>337</v>
       </c>
       <c r="AA34">
-        <v>0.99839748836760267</v>
+        <v>0.99797368969783629</v>
       </c>
       <c r="AB34">
-        <v>29.37937992728429</v>
+        <v>37.149022206335331</v>
       </c>
     </row>
   </sheetData>
@@ -10194,7 +10194,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DC2873B-1DBE-472C-92E1-6D32A391FF52}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3328AE85-653D-4F43-896B-6C25D49B89D3}">
   <dimension ref="B9:Z29"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10306,7 +10306,7 @@
         <v>489</v>
       </c>
       <c r="K11" t="s">
-        <v>410</v>
+        <v>378</v>
       </c>
       <c r="L11">
         <v>7.7363165779076795</v>
@@ -10339,7 +10339,7 @@
         <v>527</v>
       </c>
       <c r="X11" t="s">
-        <v>464</v>
+        <v>479</v>
       </c>
       <c r="Y11">
         <v>39.450749999999999</v>
@@ -10407,7 +10407,7 @@
         <v>529</v>
       </c>
       <c r="X12" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="Y12">
         <v>10.7745</v>
@@ -10442,7 +10442,7 @@
         <v>493</v>
       </c>
       <c r="K13" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="L13">
         <v>21.492626448742886</v>
@@ -10475,7 +10475,7 @@
         <v>531</v>
       </c>
       <c r="X13" t="s">
-        <v>468</v>
+        <v>483</v>
       </c>
       <c r="Y13">
         <v>38.600250000000003</v>
@@ -10543,7 +10543,7 @@
         <v>533</v>
       </c>
       <c r="X14" t="s">
-        <v>456</v>
+        <v>485</v>
       </c>
       <c r="Y14">
         <v>4.0402500000000003</v>
@@ -10578,7 +10578,7 @@
         <v>497</v>
       </c>
       <c r="K15" t="s">
-        <v>376</v>
+        <v>398</v>
       </c>
       <c r="L15">
         <v>4.0537250245901548</v>
@@ -10611,7 +10611,7 @@
         <v>535</v>
       </c>
       <c r="X15" t="s">
-        <v>458</v>
+        <v>487</v>
       </c>
       <c r="Y15">
         <v>39.321750000000002</v>
@@ -10646,7 +10646,7 @@
         <v>499</v>
       </c>
       <c r="K16" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="L16">
         <v>9.6185391844194168</v>
@@ -10679,7 +10679,7 @@
         <v>537</v>
       </c>
       <c r="X16" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="Y16">
         <v>12.592499999999999</v>
@@ -10714,7 +10714,7 @@
         <v>501</v>
       </c>
       <c r="K17" t="s">
-        <v>406</v>
+        <v>384</v>
       </c>
       <c r="L17">
         <v>20.992062966824207</v>
@@ -10747,7 +10747,7 @@
         <v>539</v>
       </c>
       <c r="X17" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="Y17">
         <v>15.871499999999999</v>
@@ -10782,7 +10782,7 @@
         <v>503</v>
       </c>
       <c r="K18" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="L18">
         <v>4.7225970155809494</v>
@@ -10815,7 +10815,7 @@
         <v>541</v>
       </c>
       <c r="X18" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="Y18">
         <v>19.04175</v>
@@ -10850,7 +10850,7 @@
         <v>505</v>
       </c>
       <c r="K19" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="L19">
         <v>9.0836490896593176</v>
@@ -10883,7 +10883,7 @@
         <v>543</v>
       </c>
       <c r="X19" t="s">
-        <v>482</v>
+        <v>470</v>
       </c>
       <c r="Y19">
         <v>28.344000000000001</v>
@@ -10918,7 +10918,7 @@
         <v>507</v>
       </c>
       <c r="K20" t="s">
-        <v>400</v>
+        <v>376</v>
       </c>
       <c r="L20">
         <v>10.618766499150132</v>
@@ -10951,7 +10951,7 @@
         <v>545</v>
       </c>
       <c r="X20" t="s">
-        <v>466</v>
+        <v>481</v>
       </c>
       <c r="Y20">
         <v>14.163</v>
@@ -10986,7 +10986,7 @@
         <v>509</v>
       </c>
       <c r="K21" t="s">
-        <v>380</v>
+        <v>402</v>
       </c>
       <c r="L21">
         <v>37.276481001553563</v>
@@ -11019,7 +11019,7 @@
         <v>547</v>
       </c>
       <c r="X21" t="s">
-        <v>462</v>
+        <v>477</v>
       </c>
       <c r="Y21">
         <v>2.0775000000000001</v>
@@ -11054,7 +11054,7 @@
         <v>511</v>
       </c>
       <c r="K22" t="s">
-        <v>390</v>
+        <v>412</v>
       </c>
       <c r="L22">
         <v>20.90644030096918</v>
@@ -11087,7 +11087,7 @@
         <v>549</v>
       </c>
       <c r="X22" t="s">
-        <v>480</v>
+        <v>468</v>
       </c>
       <c r="Y22">
         <v>9.2415000000000003</v>
@@ -11122,7 +11122,7 @@
         <v>513</v>
       </c>
       <c r="K23" t="s">
-        <v>408</v>
+        <v>386</v>
       </c>
       <c r="L23">
         <v>1.24293744829465</v>
@@ -11155,7 +11155,7 @@
         <v>551</v>
       </c>
       <c r="X23" t="s">
-        <v>486</v>
+        <v>454</v>
       </c>
       <c r="Y23">
         <v>0.97650000000000003</v>
@@ -11190,7 +11190,7 @@
         <v>515</v>
       </c>
       <c r="K24" t="s">
-        <v>412</v>
+        <v>380</v>
       </c>
       <c r="L24">
         <v>3.655060122103603</v>
@@ -11223,7 +11223,7 @@
         <v>553</v>
       </c>
       <c r="X24" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="Y24">
         <v>6.8857499999999998</v>
@@ -11258,7 +11258,7 @@
         <v>517</v>
       </c>
       <c r="K25" t="s">
-        <v>382</v>
+        <v>404</v>
       </c>
       <c r="L25">
         <v>48.450394178145253</v>
@@ -11291,7 +11291,7 @@
         <v>555</v>
       </c>
       <c r="X25" t="s">
-        <v>478</v>
+        <v>466</v>
       </c>
       <c r="Y25">
         <v>71.778000000000006</v>
@@ -11326,7 +11326,7 @@
         <v>519</v>
       </c>
       <c r="K26" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="L26">
         <v>19.948651692996549</v>
@@ -11359,7 +11359,7 @@
         <v>557</v>
       </c>
       <c r="X26" t="s">
-        <v>484</v>
+        <v>452</v>
       </c>
       <c r="Y26">
         <v>40.861499999999999</v>
@@ -11462,7 +11462,7 @@
         <v>523</v>
       </c>
       <c r="K28" t="s">
-        <v>378</v>
+        <v>400</v>
       </c>
       <c r="L28">
         <v>6.7463178806119855</v>
@@ -11495,7 +11495,7 @@
         <v>561</v>
       </c>
       <c r="X28" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="Y28">
         <v>49.423499999999997</v>
@@ -11530,7 +11530,7 @@
         <v>525</v>
       </c>
       <c r="K29" t="s">
-        <v>398</v>
+        <v>410</v>
       </c>
       <c r="L29">
         <v>9.7794224100622564</v>
@@ -11563,7 +11563,7 @@
         <v>563</v>
       </c>
       <c r="X29" t="s">
-        <v>488</v>
+        <v>474</v>
       </c>
       <c r="Y29">
         <v>48.613500000000002</v>
@@ -11578,7 +11578,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A99FF4E-C07D-43F4-ACD1-39C889CB6869}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92BF7CCB-7AA8-4C42-ADBC-F902994712F0}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13395,7 +13395,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EF24219-2739-4267-B50E-E482051CE90F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{557C0D51-BC31-4D09-87AC-80818F3E4BB1}">
   <dimension ref="B2:M15"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>